<commit_message>
adding zika virus test data
</commit_message>
<xml_diff>
--- a/example_files/zika_virus_test_metadata.xlsx
+++ b/example_files/zika_virus_test_metadata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\skasambula\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E9F4D20C-550F-4C83-B2A1-DE91B2BE7AF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A18F5AC-CBEC-4CCA-9EC6-25722A984D99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BC45BC39-EA9A-48B3-A412-1DBB9FBA7354}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="111">
   <si>
     <t>id</t>
   </si>
@@ -306,9 +306,6 @@
     <t>Kenya</t>
   </si>
   <si>
-    <t>Homosapiens</t>
-  </si>
-  <si>
     <t>test_zika_006</t>
   </si>
   <si>
@@ -364,6 +361,12 @@
   </si>
   <si>
     <t>CNR Arbovirus, CNR Arbovirus</t>
+  </si>
+  <si>
+    <t>Homo sapiens</t>
+  </si>
+  <si>
+    <t>Aedes aegypti</t>
   </si>
 </sst>
 </file>
@@ -730,7 +733,7 @@
     <col min="3" max="3" width="19.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="39.5546875" customWidth="1"/>
     <col min="5" max="5" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.21875" customWidth="1"/>
     <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -993,13 +996,13 @@
         <v>46235</v>
       </c>
       <c r="D2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F2" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:82" x14ac:dyDescent="0.3">
@@ -1013,13 +1016,13 @@
         <v>46236</v>
       </c>
       <c r="D3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F3" t="s">
-        <v>90</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:82" x14ac:dyDescent="0.3">
@@ -1036,10 +1039,10 @@
         <v>88</v>
       </c>
       <c r="E4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F4" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:82" x14ac:dyDescent="0.3">
@@ -1056,10 +1059,10 @@
         <v>88</v>
       </c>
       <c r="E5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F5" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:82" x14ac:dyDescent="0.3">
@@ -1076,15 +1079,15 @@
         <v>88</v>
       </c>
       <c r="E6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F6" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" spans="1:82" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B7" t="s">
         <v>87</v>
@@ -1093,18 +1096,18 @@
         <v>46236</v>
       </c>
       <c r="D7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F7" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8" spans="1:82" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B8" t="s">
         <v>87</v>
@@ -1113,73 +1116,73 @@
         <v>46236</v>
       </c>
       <c r="D8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F8" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:82" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C9" s="1">
         <v>46235</v>
       </c>
       <c r="D9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F9" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
     </row>
     <row r="10" spans="1:82" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C10" s="1">
         <v>46235</v>
       </c>
       <c r="D10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E10" t="s">
+        <v>108</v>
+      </c>
+      <c r="F10" t="s">
         <v>109</v>
-      </c>
-      <c r="F10" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="11" spans="1:82" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" t="s">
         <v>95</v>
-      </c>
-      <c r="B11" t="s">
-        <v>96</v>
       </c>
       <c r="C11" s="1">
         <v>46235</v>
       </c>
       <c r="D11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E11" t="s">
+        <v>108</v>
+      </c>
+      <c r="F11" t="s">
         <v>109</v>
-      </c>
-      <c r="F11" t="s">
-        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Merge example metadata files
</commit_message>
<xml_diff>
--- a/example_files/zika_virus_test_metadata.xlsx
+++ b/example_files/zika_virus_test_metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\skasambula\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mverbies/projects/dev_example_data/example_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A18F5AC-CBEC-4CCA-9EC6-25722A984D99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCE58A2A-C088-A744-A51D-4D3D4C51D59B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BC45BC39-EA9A-48B3-A412-1DBB9FBA7354}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{BC45BC39-EA9A-48B3-A412-1DBB9FBA7354}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="115">
   <si>
     <t>id</t>
   </si>
@@ -367,6 +367,18 @@
   </si>
   <si>
     <t>Aedes aegypti</t>
+  </si>
+  <si>
+    <t>Homosapiens</t>
+  </si>
+  <si>
+    <t>Kenya/zika01/2026</t>
+  </si>
+  <si>
+    <t>Kenya/zika 02/2026</t>
+  </si>
+  <si>
+    <t>Brazil/zika_10/2026-01-08</t>
   </si>
 </sst>
 </file>
@@ -429,9 +441,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -469,7 +481,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -575,7 +587,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -717,7 +729,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -726,18 +738,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FBBF866-AA12-4734-82A3-26102C461E93}">
   <dimension ref="A1:CD11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.6640625" customWidth="1"/>
     <col min="2" max="2" width="15.33203125" customWidth="1"/>
-    <col min="3" max="3" width="19.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39.5546875" customWidth="1"/>
-    <col min="5" max="5" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.21875" customWidth="1"/>
-    <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="39.5" customWidth="1"/>
+    <col min="5" max="5" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.1640625" customWidth="1"/>
+    <col min="7" max="7" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:82" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -985,7 +998,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:82" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>82</v>
       </c>
@@ -1004,8 +1017,11 @@
       <c r="F2" t="s">
         <v>109</v>
       </c>
+      <c r="Q2" t="s">
+        <v>112</v>
+      </c>
     </row>
-    <row r="3" spans="1:82" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>83</v>
       </c>
@@ -1024,8 +1040,11 @@
       <c r="F3" t="s">
         <v>110</v>
       </c>
+      <c r="Q3" t="s">
+        <v>113</v>
+      </c>
     </row>
-    <row r="4" spans="1:82" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>84</v>
       </c>
@@ -1045,7 +1064,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="5" spans="1:82" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>85</v>
       </c>
@@ -1065,7 +1084,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="6" spans="1:82" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>86</v>
       </c>
@@ -1082,10 +1101,10 @@
         <v>104</v>
       </c>
       <c r="F6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
-    <row r="7" spans="1:82" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>90</v>
       </c>
@@ -1105,7 +1124,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="8" spans="1:82" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>91</v>
       </c>
@@ -1125,7 +1144,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="9" spans="1:82" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>92</v>
       </c>
@@ -1145,7 +1164,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="10" spans="1:82" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>93</v>
       </c>
@@ -1165,7 +1184,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="11" spans="1:82" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>94</v>
       </c>
@@ -1183,6 +1202,9 @@
       </c>
       <c r="F11" t="s">
         <v>109</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>